<commit_message>
Update test samples and exception examples.
</commit_message>
<xml_diff>
--- a/examples/input/interactions/translated_SkeMel133_biorecipe_combined_10contradictions.xlsx
+++ b/examples/input/interactions/translated_SkeMel133_biorecipe_combined_10contradictions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luohaomiao/Desktop/code/violin_org/violin_cache_20250321/eval/input/interactions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luohaomiao/Desktop/code/violin_org/violin_cache_20250321/examples/input/interactions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8CB64F-026F-C247-9B8A-9E68DA9ED770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBDF7BC6-BE3C-9944-9800-E4AF47BB4F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31500" yWindow="-1860" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5975" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5974" uniqueCount="453">
   <si>
     <t>Regulator Name</t>
   </si>
@@ -1366,25 +1366,19 @@
     <t>we tested whether pi3k and akt inhibition in sw480 colon cancer cells triggered activation of src and tyrosine signaling , and if this correlated with transcriptional upregulation of dgkalpha . ++++ pi3k or akt inhibited cell cultures of sw480 cell showed increases in src activation and in total phosphotyrosine profiles .</t>
   </si>
   <si>
-    <t>erbb4</t>
-  </si>
-  <si>
-    <t>q15303</t>
-  </si>
-  <si>
-    <t>erbb</t>
-  </si>
-  <si>
-    <t>cellosaurus:cvcl_0620</t>
-  </si>
-  <si>
-    <t>cl:cl:0002327</t>
-  </si>
-  <si>
-    <t>erbb4 may execute its differentiation inducing function by dimerizing with other erbb family members and decreasing the levels of more oncogenic erbb heterodimers such as erbb3 and erbb2 [ xref_bibr ] .</t>
-  </si>
-  <si>
-    <t>pmc4353460</t>
+    <t>p49815</t>
+  </si>
+  <si>
+    <t>mtor</t>
+  </si>
+  <si>
+    <t>p42345</t>
+  </si>
+  <si>
+    <t>indeed , myc inhibits the mtor repressor tsc2 , thereby increasing mtor activity to facilitate translation through s6k and 4e-bp phosphorylation [ xref_bibr ] .</t>
+  </si>
+  <si>
+    <t>pmc4980327</t>
   </si>
 </sst>
 </file>
@@ -19997,31 +19991,34 @@
     </row>
     <row r="273" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
-        <v>448</v>
+        <v>317</v>
       </c>
       <c r="B273" t="s">
         <v>48</v>
       </c>
       <c r="D273" t="s">
-        <v>448</v>
+        <v>317</v>
       </c>
       <c r="E273" t="s">
         <v>401</v>
       </c>
       <c r="F273" t="s">
+        <v>448</v>
+      </c>
+      <c r="I273" t="s">
         <v>449</v>
-      </c>
-      <c r="I273" t="s">
-        <v>450</v>
       </c>
       <c r="J273" t="s">
         <v>48</v>
       </c>
+      <c r="L273" t="s">
+        <v>449</v>
+      </c>
       <c r="M273" t="s">
         <v>401</v>
       </c>
       <c r="N273" t="s">
-        <v>413</v>
+        <v>450</v>
       </c>
       <c r="Q273" t="s">
         <v>406</v>
@@ -20032,17 +20029,11 @@
       <c r="S273" t="s">
         <v>404</v>
       </c>
-      <c r="U273" t="s">
+      <c r="AA273" t="s">
         <v>451</v>
       </c>
-      <c r="V273" t="s">
+      <c r="AB273" t="s">
         <v>452</v>
-      </c>
-      <c r="AA273" t="s">
-        <v>453</v>
-      </c>
-      <c r="AB273" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="274" spans="1:28" x14ac:dyDescent="0.2">

</xml_diff>